<commit_message>
Stop offering the two measurements that say they are unfinished
1-2-3 point calibrations and Rate of Change of Soil Water Status both carry
"TO ADD if relevant (not yet implemented)" as their own tooltip, and both were
in the measurement dropdown producing a plausible looking number on the
display. build.py now leaves out any measurement whose tooltip says that, and
prints which ones it left out so it is never silent. The sheet already states
the status in prose, so honouring that beats keeping a second list in step.
Take the marker out of the tooltip and the measurement returns.

Also picks up the spreadsheet change that switches front_lcd on. Wetting Front
had no display option but "No visualization", so it could only produce a sketch
that showed nothing. Both configuration gaps the verifier was reporting are now
closed, and it runs clean: 256 sketches, no warnings.

CACHE_NAME bumped to v8.
</commit_message>
<xml_diff>
--- a/data/sensor_configuration.xlsx
+++ b/data/sensor_configuration.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fernandolaguna/Desktop/Low-Cost-Water-Tech/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fernandolaguna/Desktop/Low-Cost-Water-Tech/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D19A0DB1-6D99-6344-A864-6698A12AA84C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1FD22EF-CE11-FF4E-9517-F13F05D4F4F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3100" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2880" yWindow="1820" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sensors" sheetId="1" r:id="rId1"/>
@@ -838,11 +838,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color rgb="FFFFFF00"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -866,19 +861,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FFFF0000"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="6">
@@ -950,7 +945,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -967,17 +962,11 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1000,34 +989,29 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1414,7 +1398,7 @@
       </c>
     </row>
     <row r="6" spans="1:15">
-      <c r="A6" s="20"/>
+      <c r="A6" s="18"/>
       <c r="B6" s="3" t="s">
         <v>39</v>
       </c>
@@ -1444,7 +1428,7 @@
       </c>
     </row>
     <row r="7" spans="1:15">
-      <c r="A7" s="24"/>
+      <c r="A7" s="23"/>
       <c r="B7" s="3" t="s">
         <v>43</v>
       </c>
@@ -1471,7 +1455,7 @@
       </c>
     </row>
     <row r="8" spans="1:15">
-      <c r="A8" s="23"/>
+      <c r="A8" s="24"/>
       <c r="B8" s="3" t="s">
         <v>47</v>
       </c>
@@ -1497,8 +1481,8 @@
       <c r="J8" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9" t="s">
+      <c r="K8" s="8"/>
+      <c r="L8" s="8" t="s">
         <v>53</v>
       </c>
       <c r="O8" s="7" t="s">
@@ -1506,7 +1490,7 @@
       </c>
     </row>
     <row r="9" spans="1:15">
-      <c r="A9" s="23"/>
+      <c r="A9" s="24"/>
       <c r="B9" s="3" t="s">
         <v>218</v>
       </c>
@@ -1524,14 +1508,14 @@
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9" t="s">
+      <c r="K9" s="8"/>
+      <c r="L9" s="8" t="s">
         <v>219</v>
       </c>
       <c r="O9" s="7"/>
     </row>
     <row r="10" spans="1:15">
-      <c r="A10" s="23"/>
+      <c r="A10" s="24"/>
       <c r="B10" s="3" t="s">
         <v>55</v>
       </c>
@@ -1557,8 +1541,8 @@
       <c r="J10" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9" t="s">
+      <c r="K10" s="8"/>
+      <c r="L10" s="8" t="s">
         <v>53</v>
       </c>
       <c r="O10" s="7" t="s">
@@ -1604,16 +1588,16 @@
       <c r="D12" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="28" t="s">
         <v>21</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
-      <c r="J12" s="6" t="s">
+      <c r="J12" s="28" t="s">
         <v>22</v>
       </c>
       <c r="K12" s="5" t="s">
@@ -1622,18 +1606,18 @@
       <c r="L12" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="O12" s="10" t="s">
+      <c r="O12" s="9" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:15">
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="10" t="s">
         <v>67</v>
       </c>
       <c r="L13" s="5" t="s">
@@ -1641,22 +1625,22 @@
       </c>
     </row>
     <row r="14" spans="1:15" ht="15" customHeight="1">
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="E14" s="27" t="s">
+      <c r="E14" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="F14" s="28" t="s">
+      <c r="F14" s="16" t="s">
         <v>209</v>
       </c>
-      <c r="G14" s="28" t="s">
+      <c r="G14" s="16" t="s">
         <v>210</v>
       </c>
-      <c r="L14" s="29" t="s">
+      <c r="L14" s="5" t="s">
         <v>223</v>
       </c>
     </row>
@@ -1678,7 +1662,7 @@
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
-      <c r="J15" s="13" t="s">
+      <c r="J15" s="11" t="s">
         <v>203</v>
       </c>
       <c r="K15" s="5" t="s">
@@ -1693,22 +1677,22 @@
       <c r="B16" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="28" t="s">
         <v>18</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="28" t="s">
         <v>21</v>
       </c>
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="6" t="s">
+      <c r="J16" s="28" t="s">
         <v>22</v>
       </c>
       <c r="K16" s="5" t="s">
@@ -1717,7 +1701,7 @@
       <c r="L16" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="O16" s="10" t="s">
+      <c r="O16" s="9" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1726,7 +1710,7 @@
       <c r="B17" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="28" t="s">
         <v>70</v>
       </c>
       <c r="D17" s="3" t="s">
@@ -1760,9 +1744,9 @@
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="25"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="27"/>
       <c r="J18" s="3" t="s">
         <v>194</v>
       </c>
@@ -1772,7 +1756,7 @@
       <c r="L18" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="O18" s="10" t="s">
+      <c r="O18" s="9" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1806,14 +1790,14 @@
       </c>
     </row>
     <row r="20" spans="1:15">
-      <c r="A20" s="14"/>
-      <c r="B20" s="15" t="s">
+      <c r="A20" s="12"/>
+      <c r="B20" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="D20" s="14"/>
+      <c r="D20" s="12"/>
       <c r="E20" s="5" t="s">
         <v>208</v>
       </c>
@@ -1828,7 +1812,7 @@
       </c>
     </row>
     <row r="21" spans="1:15">
-      <c r="A21" s="34" t="s">
+      <c r="A21" s="22" t="s">
         <v>220</v>
       </c>
       <c r="B21" s="3" t="s">
@@ -1851,7 +1835,7 @@
       </c>
     </row>
     <row r="22" spans="1:15" ht="15.75" customHeight="1">
-      <c r="A22" s="14"/>
+      <c r="A22" s="12"/>
       <c r="B22" s="3" t="s">
         <v>78</v>
       </c>
@@ -1872,10 +1856,10 @@
       </c>
     </row>
     <row r="23" spans="1:15" ht="15.75" customHeight="1">
-      <c r="A23" s="14"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
+      <c r="A23" s="12"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
     </row>
     <row r="24" spans="1:15" ht="15.75" customHeight="1"/>
     <row r="25" spans="1:15" ht="15.75" customHeight="1"/>
@@ -2900,7 +2884,7 @@
       <c r="H1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="31" t="s">
+      <c r="I1" s="2" t="s">
         <v>212</v>
       </c>
     </row>
@@ -3032,64 +3016,64 @@
       </c>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="11"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
+      <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
       <c r="H7" s="5"/>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="10">
         <v>0</v>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="10">
         <v>239</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="10">
         <v>0</v>
       </c>
-      <c r="H8" s="16" t="s">
+      <c r="H8" s="14" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="10">
         <v>0</v>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="10">
         <v>200</v>
       </c>
-      <c r="G9" s="11">
+      <c r="G9" s="10">
         <v>0</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="14" t="s">
         <v>15</v>
       </c>
     </row>
@@ -3123,223 +3107,223 @@
       <c r="A11" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="15">
         <v>0</v>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="15">
         <v>1023</v>
       </c>
-      <c r="G11" s="17">
+      <c r="G11" s="15">
         <v>600</v>
       </c>
-      <c r="H11" s="16" t="s">
+      <c r="H11" s="14" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15" customHeight="1">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="19">
         <v>0</v>
       </c>
-      <c r="F12" s="21">
+      <c r="F12" s="19">
         <v>1023</v>
       </c>
-      <c r="G12" s="21">
+      <c r="G12" s="19">
         <v>450</v>
       </c>
-      <c r="H12" s="22" t="s">
+      <c r="H12" s="20" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15" customHeight="1">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="C13" s="19" t="s">
         <v>197</v>
       </c>
-      <c r="E13" s="21">
+      <c r="E13" s="19">
         <v>0</v>
       </c>
-      <c r="F13" s="21">
+      <c r="F13" s="19">
         <v>1023</v>
       </c>
-      <c r="G13" s="21">
+      <c r="G13" s="19">
         <v>350</v>
       </c>
-      <c r="H13" s="22" t="s">
+      <c r="H13" s="20" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15" customHeight="1">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="E14" s="21">
+      <c r="E14" s="19">
         <v>0</v>
       </c>
-      <c r="F14" s="21">
+      <c r="F14" s="19">
         <v>200</v>
       </c>
-      <c r="G14" s="21">
+      <c r="G14" s="19">
         <v>15</v>
       </c>
-      <c r="H14" s="22" t="s">
+      <c r="H14" s="20" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15" customHeight="1">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="E15" s="21">
+      <c r="E15" s="19">
         <v>0</v>
       </c>
-      <c r="F15" s="21">
+      <c r="F15" s="19">
         <v>200</v>
       </c>
-      <c r="G15" s="21">
+      <c r="G15" s="19">
         <v>40</v>
       </c>
-      <c r="H15" s="22" t="s">
+      <c r="H15" s="20" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15" customHeight="1">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="19" t="s">
         <v>201</v>
       </c>
-      <c r="E16" s="21">
+      <c r="E16" s="19">
         <v>0</v>
       </c>
-      <c r="F16" s="21">
+      <c r="F16" s="19">
         <v>1023</v>
       </c>
-      <c r="G16" s="21">
+      <c r="G16" s="19">
         <v>400</v>
       </c>
-      <c r="H16" s="16" t="s">
+      <c r="H16" s="14" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15" customHeight="1">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="B17" s="21" t="s">
+      <c r="B17" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="C17" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="E17" s="21">
+      <c r="E17" s="19">
         <v>0</v>
       </c>
-      <c r="F17" s="21">
+      <c r="F17" s="19">
         <v>239</v>
       </c>
-      <c r="G17" s="21">
+      <c r="G17" s="19">
         <v>239</v>
       </c>
-      <c r="H17" s="16" t="s">
+      <c r="H17" s="14" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15" customHeight="1">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="E18" s="21">
+      <c r="E18" s="19">
         <v>0</v>
       </c>
-      <c r="F18" s="21">
+      <c r="F18" s="19">
         <v>239</v>
       </c>
-      <c r="G18" s="21">
+      <c r="G18" s="19">
         <v>239</v>
       </c>
-      <c r="H18" s="16" t="s">
+      <c r="H18" s="14" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15" customHeight="1">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="B19" s="21" t="s">
+      <c r="B19" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="C19" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="E19" s="21">
+      <c r="E19" s="19">
         <v>0</v>
       </c>
-      <c r="F19" s="21">
+      <c r="F19" s="19">
         <v>239</v>
       </c>
-      <c r="G19" s="21">
+      <c r="G19" s="19">
         <v>0</v>
       </c>
-      <c r="H19" s="16" t="s">
+      <c r="H19" s="14" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15" customHeight="1">
-      <c r="A20" s="26" t="s">
+      <c r="A20" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="30" t="s">
+      <c r="B20" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="C20" s="30" t="s">
+      <c r="C20" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="D20" s="32" t="s">
+      <c r="D20" s="21" t="s">
         <v>213</v>
       </c>
       <c r="G20" s="5" t="s">
@@ -3350,13 +3334,13 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A21" s="26" t="s">
+      <c r="A21" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="B21" s="30" t="s">
+      <c r="B21" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="C21" s="30" t="s">
+      <c r="C21" s="19" t="s">
         <v>211</v>
       </c>
       <c r="D21" s="5" t="s">
@@ -3370,94 +3354,94 @@
       </c>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A22" s="26" t="s">
+      <c r="A22" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="B22" s="30" t="s">
+      <c r="B22" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="C22" s="32" t="s">
+      <c r="C22" s="21" t="s">
         <v>216</v>
       </c>
-      <c r="E22" s="28">
+      <c r="E22" s="16">
         <v>0</v>
       </c>
-      <c r="F22" s="28">
+      <c r="F22" s="16">
         <v>239</v>
       </c>
-      <c r="G22" s="28">
+      <c r="G22" s="16">
         <v>23</v>
       </c>
-      <c r="H22" s="33" t="s">
+      <c r="H22" s="14" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A23" s="26" t="s">
+      <c r="A23" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="B23" s="30" t="s">
+      <c r="B23" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="16" t="s">
         <v>217</v>
       </c>
-      <c r="E23" s="28">
+      <c r="E23" s="16">
         <v>0</v>
       </c>
-      <c r="F23" s="28">
+      <c r="F23" s="16">
         <v>239</v>
       </c>
-      <c r="G23" s="28">
+      <c r="G23" s="16">
         <v>65</v>
       </c>
-      <c r="H23" s="33" t="s">
+      <c r="H23" s="14" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A24" s="26" t="s">
+      <c r="A24" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="B24" s="30" t="s">
+      <c r="B24" s="19" t="s">
         <v>209</v>
       </c>
       <c r="C24" t="s">
         <v>216</v>
       </c>
-      <c r="E24" s="28">
+      <c r="E24" s="16">
         <v>0</v>
       </c>
-      <c r="F24" s="28">
+      <c r="F24" s="16">
         <v>239</v>
       </c>
-      <c r="G24" s="28">
+      <c r="G24" s="16">
         <v>23</v>
       </c>
-      <c r="H24" s="33" t="s">
+      <c r="H24" s="14" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A25" s="26" t="s">
+      <c r="A25" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="B25" s="30" t="s">
+      <c r="B25" s="19" t="s">
         <v>210</v>
       </c>
       <c r="C25" t="s">
         <v>217</v>
       </c>
-      <c r="E25" s="28">
+      <c r="E25" s="16">
         <v>0</v>
       </c>
-      <c r="F25" s="28">
+      <c r="F25" s="16">
         <v>239</v>
       </c>
-      <c r="G25" s="28">
+      <c r="G25" s="16">
         <v>65</v>
       </c>
-      <c r="H25" s="33" t="s">
+      <c r="H25" s="14" t="s">
         <v>23</v>
       </c>
     </row>
@@ -5602,122 +5586,122 @@
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="10" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="10" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="10" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="10" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="10" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="10" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="10" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="10" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="10" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="10" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15.75" customHeight="1">
-      <c r="B21" s="18"/>
+      <c r="B21" s="16"/>
     </row>
     <row r="22" spans="1:2" ht="15.75" customHeight="1">
-      <c r="B22" s="18"/>
+      <c r="B22" s="16"/>
     </row>
     <row r="23" spans="1:2" ht="15.75" customHeight="1"/>
     <row r="24" spans="1:2" ht="15.75" customHeight="1"/>
@@ -6814,55 +6798,55 @@
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="10" t="s">
         <v>186</v>
       </c>
-      <c r="D8" s="19" t="b">
-        <v>0</v>
+      <c r="D8" s="17" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:4">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="17" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="D10" s="18" t="b">
+      <c r="D10" s="16" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15" customHeight="1">
-      <c r="A11" s="26" t="s">
+      <c r="A11" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="C11" s="10" t="s">
         <v>222</v>
       </c>
       <c r="D11" s="5" t="s">
@@ -6870,13 +6854,13 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="15" customHeight="1">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="10" t="s">
         <v>228</v>
       </c>
-      <c r="C12" s="26" t="s">
+      <c r="C12" s="10" t="s">
         <v>224</v>
       </c>
       <c r="D12" t="b">

</xml_diff>

<commit_message>
Restore the ports edits, and warn when Excel is holding the sheet
The ports sheet lost its active column and its digital rows again: Excel still
had the file open and wrote its own copy back over them. Reapplied and verified
by reading the file straight back.

build.py now looks for the ~$ lock file Excel leaves beside anything it has
open, and says plainly that Excel will overwrite script edits when it saves or
quits. This is the second time it happened; a warning is cheaper than losing
the edits a third time.
</commit_message>
<xml_diff>
--- a/data/sensor_configuration.xlsx
+++ b/data/sensor_configuration.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fernandolaguna/Desktop/Low-Cost-Water-Tech/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1FD22EF-CE11-FF4E-9517-F13F05D4F4F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2FA4B31-0D8B-9649-9855-695F402761F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2880" yWindow="1820" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="3180" yWindow="3400" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sensors" sheetId="1" r:id="rId1"/>
@@ -691,9 +691,32 @@
     <t>rate_lcd</t>
   </si>
   <si>
+    <t>Flow rate</t>
+  </si>
+  <si>
+    <t>Displays the flow rate between 2 sensors</t>
+  </si>
+  <si>
+    <t>wm_state_lcd</t>
+  </si>
+  <si>
+    <t>Displays the state at which the soils seems to be for the Watermark sensors</t>
+  </si>
+  <si>
+    <t>Displays the general state at which soil seems to be for the capacitive sensors</t>
+  </si>
+  <si>
+    <t>wm_state_lcd|bar|transformed_lcd</t>
+  </si>
+  <si>
+    <t>State: Very Dry, Dry, or Wet</t>
+  </si>
+  <si>
+    <t>State: Dry plant stressed, Irrigation range, or Saturation</t>
+  </si>
+  <si>
     <r>
       <rPr>
-        <b/>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
@@ -704,7 +727,6 @@
     </r>
     <r>
       <rPr>
-        <b/>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri (Body)"/>
@@ -712,36 +734,12 @@
       <t>rrometer Soil Temperature Sensor (200TS)</t>
     </r>
   </si>
-  <si>
-    <t>Flow rate</t>
-  </si>
-  <si>
-    <t>Displays the flow rate between 2 sensors</t>
-  </si>
-  <si>
-    <t>wm_state_lcd</t>
-  </si>
-  <si>
-    <t>Displays the state at which the soils seems to be for the Watermark sensors</t>
-  </si>
-  <si>
-    <t>Displays the general state at which soil seems to be for the capacitive sensors</t>
-  </si>
-  <si>
-    <t>wm_state_lcd|bar|transformed_lcd</t>
-  </si>
-  <si>
-    <t>State: Very Dry, Dry, or Wet</t>
-  </si>
-  <si>
-    <t>State: Dry plant stressed, Irrigation range, or Saturation</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -848,24 +846,15 @@
       <name val="-webkit-standard"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri (Body)"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="3"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri (Body)"/>
     </font>
   </fonts>
   <fills count="2">
@@ -945,7 +934,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -990,7 +979,6 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1003,13 +991,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1428,7 +1416,7 @@
       </c>
     </row>
     <row r="7" spans="1:15">
-      <c r="A7" s="23"/>
+      <c r="A7" s="22"/>
       <c r="B7" s="3" t="s">
         <v>43</v>
       </c>
@@ -1455,7 +1443,7 @@
       </c>
     </row>
     <row r="8" spans="1:15">
-      <c r="A8" s="24"/>
+      <c r="A8" s="23"/>
       <c r="B8" s="3" t="s">
         <v>47</v>
       </c>
@@ -1490,7 +1478,7 @@
       </c>
     </row>
     <row r="9" spans="1:15">
-      <c r="A9" s="24"/>
+      <c r="A9" s="23"/>
       <c r="B9" s="3" t="s">
         <v>218</v>
       </c>
@@ -1515,7 +1503,7 @@
       <c r="O9" s="7"/>
     </row>
     <row r="10" spans="1:15">
-      <c r="A10" s="24"/>
+      <c r="A10" s="23"/>
       <c r="B10" s="3" t="s">
         <v>55</v>
       </c>
@@ -1588,23 +1576,23 @@
       <c r="D12" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E12" s="28" t="s">
+      <c r="E12" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="F12" s="28" t="s">
+      <c r="F12" s="27" t="s">
         <v>21</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
-      <c r="J12" s="28" t="s">
+      <c r="J12" s="27" t="s">
         <v>22</v>
       </c>
       <c r="K12" s="5" t="s">
         <v>23</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="O12" s="9" t="s">
         <v>65</v>
@@ -1614,7 +1602,7 @@
       <c r="B13" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="28" t="s">
         <v>66</v>
       </c>
       <c r="D13" s="10" t="s">
@@ -1641,7 +1629,7 @@
         <v>210</v>
       </c>
       <c r="L14" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="15" spans="1:15">
@@ -1677,29 +1665,29 @@
       <c r="B16" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="28" t="s">
+      <c r="C16" s="27" t="s">
         <v>18</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E16" s="28" t="s">
+      <c r="E16" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="F16" s="28" t="s">
+      <c r="F16" s="27" t="s">
         <v>21</v>
       </c>
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="28" t="s">
+      <c r="J16" s="27" t="s">
         <v>22</v>
       </c>
       <c r="K16" s="5" t="s">
         <v>23</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="O16" s="9" t="s">
         <v>65</v>
@@ -1710,7 +1698,7 @@
       <c r="B17" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="27" t="s">
         <v>70</v>
       </c>
       <c r="D17" s="3" t="s">
@@ -1743,10 +1731,10 @@
         <v>74</v>
       </c>
       <c r="E18" s="3"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="27"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="25"/>
+      <c r="I18" s="26"/>
       <c r="J18" s="3" t="s">
         <v>194</v>
       </c>
@@ -1808,12 +1796,12 @@
         <v>210</v>
       </c>
       <c r="L20" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="21" spans="1:15">
-      <c r="A21" s="22" t="s">
-        <v>220</v>
+      <c r="A21" s="5" t="s">
+        <v>228</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>73</v>
@@ -6760,10 +6748,10 @@
         <v>29</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>115</v>
@@ -6844,10 +6832,10 @@
         <v>219</v>
       </c>
       <c r="B11" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>221</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>222</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>187</v>
@@ -6855,13 +6843,13 @@
     </row>
     <row r="12" spans="1:4" ht="15" customHeight="1">
       <c r="A12" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>223</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>224</v>
       </c>
       <c r="D12" t="b">
         <v>1</v>

</xml_diff>